<commit_message>
feat(openenum): add is_open boolean slot to enum expressions
Add an is_open slot to enum_expression, allowing an enumeration to be
declared open so data values outside the permissible value set are
allowed. Includes tests.

Regenerate project artefacts from the updated schema, and exclude
gen-project outputs (trailing whitespace / end-of-file-fixer) from
pre-commit since the generators emit formatting we don't control.
</commit_message>
<xml_diff>
--- a/linkml_model/excel/meta.xlsx
+++ b/linkml_model/excel/meta.xlsx
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K1"/>
+  <dimension ref="A1:L1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -491,30 +491,35 @@
       </c>
       <c r="F1" t="inlineStr">
         <is>
+          <t>is_open</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
           <t>include</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>minus</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>inherits</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>reachable_from</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>matches</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>concepts</t>
         </is>
@@ -536,7 +541,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K1"/>
+  <dimension ref="A1:L1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -567,30 +572,35 @@
       </c>
       <c r="F1" t="inlineStr">
         <is>
+          <t>is_open</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
           <t>include</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>minus</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>inherits</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>reachable_from</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>matches</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>concepts</t>
         </is>
@@ -612,7 +622,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BJ1"/>
+  <dimension ref="A1:BK1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -648,280 +658,285 @@
       </c>
       <c r="G1" t="inlineStr">
         <is>
+          <t>is_open</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
           <t>include</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>minus</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>inherits</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>reachable_from</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>matches</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>concepts</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>is_a</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>abstract</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>mixin</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>mixins</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>apply_to</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>values_from</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>string_serialization</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>id_prefixes</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>id_prefixes_are_closed</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>definition_uri</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>local_names</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>conforms_to</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="AA1" t="inlineStr">
         <is>
           <t>implements</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AB1" t="inlineStr">
         <is>
           <t>instantiates</t>
         </is>
       </c>
-      <c r="AB1" t="inlineStr">
+      <c r="AC1" t="inlineStr">
         <is>
           <t>extensions</t>
         </is>
       </c>
-      <c r="AC1" t="inlineStr">
+      <c r="AD1" t="inlineStr">
         <is>
           <t>annotations</t>
         </is>
       </c>
-      <c r="AD1" t="inlineStr">
+      <c r="AE1" t="inlineStr">
         <is>
           <t>description</t>
         </is>
       </c>
-      <c r="AE1" t="inlineStr">
+      <c r="AF1" t="inlineStr">
         <is>
           <t>alt_descriptions</t>
         </is>
       </c>
-      <c r="AF1" t="inlineStr">
+      <c r="AG1" t="inlineStr">
         <is>
           <t>title</t>
         </is>
       </c>
-      <c r="AG1" t="inlineStr">
+      <c r="AH1" t="inlineStr">
         <is>
           <t>deprecated</t>
         </is>
       </c>
-      <c r="AH1" t="inlineStr">
+      <c r="AI1" t="inlineStr">
         <is>
           <t>todos</t>
         </is>
       </c>
-      <c r="AI1" t="inlineStr">
+      <c r="AJ1" t="inlineStr">
         <is>
           <t>notes</t>
         </is>
       </c>
-      <c r="AJ1" t="inlineStr">
+      <c r="AK1" t="inlineStr">
         <is>
           <t>comments</t>
         </is>
       </c>
-      <c r="AK1" t="inlineStr">
+      <c r="AL1" t="inlineStr">
         <is>
           <t>examples</t>
         </is>
       </c>
-      <c r="AL1" t="inlineStr">
+      <c r="AM1" t="inlineStr">
         <is>
           <t>in_subset</t>
         </is>
       </c>
-      <c r="AM1" t="inlineStr">
+      <c r="AN1" t="inlineStr">
         <is>
           <t>from_schema</t>
         </is>
       </c>
-      <c r="AN1" t="inlineStr">
+      <c r="AO1" t="inlineStr">
         <is>
           <t>imported_from</t>
         </is>
       </c>
-      <c r="AO1" t="inlineStr">
+      <c r="AP1" t="inlineStr">
         <is>
           <t>source</t>
         </is>
       </c>
-      <c r="AP1" t="inlineStr">
+      <c r="AQ1" t="inlineStr">
         <is>
           <t>in_language</t>
         </is>
       </c>
-      <c r="AQ1" t="inlineStr">
+      <c r="AR1" t="inlineStr">
         <is>
           <t>see_also</t>
         </is>
       </c>
-      <c r="AR1" t="inlineStr">
+      <c r="AS1" t="inlineStr">
         <is>
           <t>deprecated element has exact replacement</t>
         </is>
       </c>
-      <c r="AS1" t="inlineStr">
+      <c r="AT1" t="inlineStr">
         <is>
           <t>deprecated element has possible replacement</t>
         </is>
       </c>
-      <c r="AT1" t="inlineStr">
+      <c r="AU1" t="inlineStr">
         <is>
           <t>aliases</t>
         </is>
       </c>
-      <c r="AU1" t="inlineStr">
+      <c r="AV1" t="inlineStr">
         <is>
           <t>structured_aliases</t>
         </is>
       </c>
-      <c r="AV1" t="inlineStr">
+      <c r="AW1" t="inlineStr">
         <is>
           <t>mappings</t>
         </is>
       </c>
-      <c r="AW1" t="inlineStr">
+      <c r="AX1" t="inlineStr">
         <is>
           <t>exact mappings</t>
         </is>
       </c>
-      <c r="AX1" t="inlineStr">
+      <c r="AY1" t="inlineStr">
         <is>
           <t>close mappings</t>
         </is>
       </c>
-      <c r="AY1" t="inlineStr">
+      <c r="AZ1" t="inlineStr">
         <is>
           <t>related mappings</t>
         </is>
       </c>
-      <c r="AZ1" t="inlineStr">
+      <c r="BA1" t="inlineStr">
         <is>
           <t>narrow mappings</t>
         </is>
       </c>
-      <c r="BA1" t="inlineStr">
+      <c r="BB1" t="inlineStr">
         <is>
           <t>broad mappings</t>
         </is>
       </c>
-      <c r="BB1" t="inlineStr">
+      <c r="BC1" t="inlineStr">
         <is>
           <t>created_by</t>
         </is>
       </c>
-      <c r="BC1" t="inlineStr">
+      <c r="BD1" t="inlineStr">
         <is>
           <t>contributors</t>
         </is>
       </c>
-      <c r="BD1" t="inlineStr">
+      <c r="BE1" t="inlineStr">
         <is>
           <t>created_on</t>
         </is>
       </c>
-      <c r="BE1" t="inlineStr">
+      <c r="BF1" t="inlineStr">
         <is>
           <t>last_updated_on</t>
         </is>
       </c>
-      <c r="BF1" t="inlineStr">
+      <c r="BG1" t="inlineStr">
         <is>
           <t>modified_by</t>
         </is>
       </c>
-      <c r="BG1" t="inlineStr">
+      <c r="BH1" t="inlineStr">
         <is>
           <t>status</t>
         </is>
       </c>
-      <c r="BH1" t="inlineStr">
+      <c r="BI1" t="inlineStr">
         <is>
           <t>rank</t>
         </is>
       </c>
-      <c r="BI1" t="inlineStr">
+      <c r="BJ1" t="inlineStr">
         <is>
           <t>categories</t>
         </is>
       </c>
-      <c r="BJ1" t="inlineStr">
+      <c r="BK1" t="inlineStr">
         <is>
           <t>keywords</t>
         </is>

</xml_diff>